<commit_message>
Data update: 2026-10-06 17:13 UTC
</commit_message>
<xml_diff>
--- a/tracking_sheet_hiddenhistory.xlsx
+++ b/tracking_sheet_hiddenhistory.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -544,7 +544,69 @@
           <t>Success</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-10-06 17:13 UTC</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>orj6xNSQzX4</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Vanished Colony Mystery: Dark Secrets of America Exposed</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>hidden history, forgotten colony, American history mystery, dark secrets, historical mysteries, vanished settlements, underground US history, secret government, archaeological mystery, historical investigation, US hidden history, British history, Australian history, Canadian history, Swiss history</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Data update: 2026-10-06 17:30 UTC
</commit_message>
<xml_diff>
--- a/tracking_sheet_hiddenhistory.xlsx
+++ b/tracking_sheet_hiddenhistory.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:M4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -606,7 +606,65 @@
           <t>Success</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-10-06 17:30 UTC</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>orj6xNSQzX4</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Forgotten Island: US Hidden Histories Revealed</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Forgotten Island, Hidden US History, Untold American History, British Influence in America, African American Pioneers, Historical Mysteries, Dark History, Historical Secrets, Colonial America, Lost Civilizations, Ancient Maps, Historical Archives, Cultural Heritage, Secret Histories, National History</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Data update: 2026-10-06 19:58 UTC
</commit_message>
<xml_diff>
--- a/tracking_sheet_hiddenhistory.xlsx
+++ b/tracking_sheet_hiddenhistory.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:M5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -664,7 +664,65 @@
           <t>Success</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-10-06 19:58 UTC</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>orj6xNSQzX4</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Hidden U.S. History Exposed: 3 Shocking Secrets</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Hidden History, Untold History, Forgotten History, American History, Secret Alliances, Historical Mysteries, Dark History Facts, US History Secrets, Pioneers, World War History, Cultural Heritage, Historical Exploration, Untold Stories, History Buffs, Educational Video</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>+1</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Data update: 2026-10-09 19:59 UTC
</commit_message>
<xml_diff>
--- a/tracking_sheet_hiddenhistory.xlsx
+++ b/tracking_sheet_hiddenhistory.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -722,7 +722,297 @@
           <t>Success</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-10-09 19:59 UTC</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ivWbJvESQzU</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Hidden Island Secrets: Untold US History Revealed</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>hidden history, untold US history, forgotten island, historical mysteries, dark history facts, secret experiments, American folklore, history reveal, cultural heritage, US hidden stories, Australia history, Canada history, UK history, Switzerland history, Norway history</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>N/A (pehli update)</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>N/A (pehli update)</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>N/A (pehli update)</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-10-09 19:59 UTC</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>oIqhWzf2xuA</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Lost 1904 Railroad: America's Hidden Mystery</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>1904 railroad mystery, hidden US history, historical mystery, unexplained disappearance, railroad history, lost train, unsolved historical mystery, American history secrets, history short, short documentary</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>N/A (pehli update)</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>N/A (pehli update)</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>N/A (pehli update)</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-10-09 19:59 UTC</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>6WctPm4ucMQ</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Secret U.S. Islands: Dark History Exposed in 60 Seconds</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Hidden US History, Secret Islands, Dark History, Untold US Stories, Historical Mysteries, World War II Secrets, 60 Second History, US Forgotten History, Historical Secrets, Hidden Wartime Bases, Island Mysteries, US Dark Secrets, Historical Short, Secret History Revealed, Shorts History</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>N/A (pehli update)</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>N/A (pehli update)</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>N/A (pehli update)</t>
+        </is>
+      </c>
+      <c r="K8" t="n">
+        <v>45</v>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-10-09 19:59 UTC</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>8n5OmnJcM_U</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Mystery of the Hidden U.S. Island: Dark Secrets Unveiled</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>hidden history, untold US history, historical mystery, secret islands, dark history, American secrets, US military history, indigenous history, historical intrigue, shorts, history reveal, US secrets, history mystery, historical facts, shorts video</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>N/A (pehli update)</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>N/A (pehli update)</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>N/A (pehli update)</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
+        <v>19</v>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-10-09 19:59 UTC</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>n21ry2t65_k</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Vanished Colony Mystery: Dark US Secret Exposed</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Vanished Colony, Hidden US History, Historical Mystery, Unsolved History, Dark Secret, Lost Colony, American History, Untold Stories, Mysterious Disappearance, Secret Government, History Short, US Secrets, Australia History, Canada History, UK History, Switzerland History, Norway History</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>125</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>N/A (pehli update)</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>N/A (pehli update)</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>N/A (pehli update)</t>
+        </is>
+      </c>
+      <c r="K10" t="n">
+        <v>8</v>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Data update: 2026-10-12 22:23 UTC
</commit_message>
<xml_diff>
--- a/tracking_sheet_hiddenhistory.xlsx
+++ b/tracking_sheet_hiddenhistory.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M10"/>
+  <dimension ref="A1:M15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1012,7 +1012,297 @@
           <t>Success</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-10-12 22:23 UTC</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>PSq-SPjXrug</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Hidden U.S. Secrets: Untold History Exposed</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>hidden history, untold history, forgotten history, historical mysteries, dark history facts, U.S. secrets, American history, history reveal, secret service history, civil rights history, indigenous history, historical secrets, history documentary, short history video, history mysteries</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>N/A (pehli update)</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>N/A (pehli update)</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>N/A (pehli update)</t>
+        </is>
+      </c>
+      <c r="K11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-10-12 22:23 UTC</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ivWbJvESQzU</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Unveiled: America’s Hidden History Exposed</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Hidden US History, Untold History, American Secrets, Historical Mysteries, Forgotten US Events, Secret Islands, Dark History Facts, America Revealed, History Shorts, US Hidden Truths</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>102</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>+102</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K12" t="n">
+        <v>29</v>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-10-12 22:23 UTC</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>oIqhWzf2xuA</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>1904 Railroad Mystery: America's Lost Line Exposed</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>1904 railroad, lost railroad, hidden history, American mystery, historical secrets, forgotten US history, railway mystery, dark history facts, US history reveal, underground rail, railway conspiracy, historical mystery, secret tracks, unexplained disappearance, history short</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>2</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>+2</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K13" t="n">
+        <v>35</v>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-10-12 22:23 UTC</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>6WctPm4ucMQ</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Hidden US Islands: Dark Secrets Revealed in 60 Seconds</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Hidden US history, Secret islands, Untold American stories, Historical mysteries, Dark history, Forgotten US history, Railroad secrets, Military experiments, US government secrets, 60 second history, Shorts, American lore, History reveal, US hidden gems, Mysterious US locations</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>4</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>+3</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K14" t="n">
+        <v>35</v>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-10-12 22:23 UTC</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>8n5OmnJcM_U</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Hidden U.S. Island Mystery: Dark Secrets Uncovered</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>hidden U.S. island, American history mystery, untold U.S. history, dark secrets, historical mysteries, forgotten U.S. sites, military secrets, lost communities, 1904 railroad mystery, America's hidden past, history short, shorts, YouTube Shorts, high CPM content, US history</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>2</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>+1</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K15" t="n">
+        <v>9</v>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Data update: 2026-10-15 18:53 UTC
</commit_message>
<xml_diff>
--- a/tracking_sheet_hiddenhistory.xlsx
+++ b/tracking_sheet_hiddenhistory.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M15"/>
+  <dimension ref="A1:M20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1302,7 +1302,297 @@
           <t>Success</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-10-15 18:52 UTC</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>PSq-SPjXrug</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Secret U.S. History Exposed: Hidden Truths Revealed</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Hidden History, Untold History, Forgotten History, Historical Mysteries, Dark History Facts, US Secrets, Secret History, History Revealed, Historical Mysteries, Hidden Truths, Untold US Stories, Dark US History, History Shorts, History YouTube Shorts, American Secrets</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>+0</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K16" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-10-15 18:53 UTC</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>ivWbJvESQzU</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Hidden U.S. Secrets Uncovered: Dark Past Revealed</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>hidden history, untold history, forgotten history, historical mysteries, dark history facts, US secrets, American history, history reveal, secret societies, historical truth, dark past, history short, US hidden truths, history facts, history documentary</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>137</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>+35</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K17" t="n">
+        <v>30</v>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-10-15 18:53 UTC</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>oIqhWzf2xuA</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Lost 1904 Railroad: America’s Hidden Tragedy Revealed</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>1904 railroad mystery, forgotten history, historical mysteries, dark history facts, hidden US history, railroad secrets, mystery short, US rail history, untold history, history short, railway mystery, history reveal, lost railroad, historical investigation, shorts history</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>2</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>+0</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K18" t="n">
+        <v>35</v>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-10-15 18:53 UTC</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>6WctPm4ucMQ</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Secret U.S. Islands: Dark History Unveiled in 60s</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>hidden history, untold history, forgotten history, historical mysteries, dark history facts, US history secrets, island mysteries, WWII espionage, indigenous stories, history short, shorts, historical revelations, secret islands, dark past, history facts</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>6</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>+2</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K19" t="n">
+        <v>19</v>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-10-15 18:53 UTC</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>8n5OmnJcM_U</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Secret U.S. Island Mystery: Dark Past Exposed</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>hidden history, untold history, forgotten history, historical mysteries, dark history facts, U.S. secrets, island mystery, American history, secret island, history reveal, dark past, hidden past, forgotten U.S. island, historical mystery short, dark history</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>2</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>+0</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K20" t="n">
+        <v>9</v>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>